<commit_message>
Uploaded updated files 01 till 10
Uploaded files 01 till 10 with updated common rules tab
</commit_message>
<xml_diff>
--- a/input/attachments/ig-assets/IPS_FHIR_to_CDISC_SDTM/01_StructureDefinition-Patient-uv-ips_to_SDTM.xlsx
+++ b/input/attachments/ig-assets/IPS_FHIR_to_CDISC_SDTM/01_StructureDefinition-Patient-uv-ips_to_SDTM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29406"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdisc-my.sharepoint.com/personal/rbaker_cdisc_org/Documents/1 Real World Data - RWD/1_XSHARE/Spreadsheets for project/IPS FHIR 1.1.0 to SDTMIG 3.4_2024-Nov/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="209" documentId="8_{07E7A70B-A1C5-49B3-94EF-8B7DCCC817C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2806BC15-2B66-44F0-B521-23952C918092}"/>
+  <xr:revisionPtr revIDLastSave="211" documentId="8_{07E7A70B-A1C5-49B3-94EF-8B7DCCC817C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{961E2F94-242A-4279-BB97-040459D3FA02}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-21465" yWindow="4905" windowWidth="19635" windowHeight="9960" firstSheet="2" activeTab="2" xr2:uid="{0620F808-081D-40E1-8012-54719B194FAA}"/>
+    <workbookView minimized="1" xWindow="-21465" yWindow="4905" windowWidth="19635" windowHeight="9960" firstSheet="2" activeTab="5" xr2:uid="{0620F808-081D-40E1-8012-54719B194FAA}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="6" r:id="rId1"/>
@@ -1658,8 +1658,7 @@
     <t xml:space="preserve">CDISC SDTM Study Identifier/STUDYID </t>
   </si>
   <si>
-    <t xml:space="preserve">For each clinical research study, populate the STUDYID variable with a default value "RWDTOSDTM-YYYYMMDD" where the date is the date on which the FHIR dataset was converted to create SDTM datasets.
-</t>
+    <t>In case there is no FHIR study ID (ResearchStudy or ResearchDefinition) available for the patient for which the immunization data is mapped, populate the STUDYID variable with a default value "RWDTOSDTM-YYYYMMDD" where the date is the date on which the FHIR dataset was converted to create SDTM datasets.</t>
   </si>
   <si>
     <t xml:space="preserve">Study Identifier/STUDYID is a variable in CDISC Demographics domain that is a unique identifier for a study. STUDYID is used as a key in all CDISC SDTM datasets.
@@ -1994,7 +1993,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -2077,6 +2076,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2345,7 +2351,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2513,6 +2519,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -16738,14 +16747,14 @@
         <v>497</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="57.6">
+    <row r="5" spans="1:4" ht="57.75">
       <c r="A5" s="32">
         <v>3</v>
       </c>
       <c r="B5" s="32" t="s">
         <v>498</v>
       </c>
-      <c r="C5" s="36" t="s">
+      <c r="C5" s="64" t="s">
         <v>499</v>
       </c>
       <c r="D5" s="30" t="s">
@@ -16961,8 +16970,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100699A48AB9E19DA4AB64847A071655FFB" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9c43450b8c34e20acaf1756fc6612395">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a46baf18-fe18-4a25-9dd7-6596c31699af" xmlns:ns3="526f0e77-c4a1-4bb9-a981-799c4b6cfc2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0a2045bb9c165ab785731dcc392b30c8" ns2:_="" ns3:_="">
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="526f0e77-c4a1-4bb9-a981-799c4b6cfc2b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a46baf18-fe18-4a25-9dd7-6596c31699af">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100699A48AB9E19DA4AB64847A071655FFB" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fb735b3d8e016bb6466dda22f76823b1">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a46baf18-fe18-4a25-9dd7-6596c31699af" xmlns:ns3="526f0e77-c4a1-4bb9-a981-799c4b6cfc2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="47d37a05d05a9fe6c5dd27e72eaf287f" ns2:_="" ns3:_="">
     <xsd:import namespace="a46baf18-fe18-4a25-9dd7-6596c31699af"/>
     <xsd:import namespace="526f0e77-c4a1-4bb9-a981-799c4b6cfc2b"/>
     <xsd:element name="properties">
@@ -16985,6 +17014,7 @@
                 <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -17052,6 +17082,11 @@
     <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -17195,28 +17230,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="526f0e77-c4a1-4bb9-a981-799c4b6cfc2b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a46baf18-fe18-4a25-9dd7-6596c31699af">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48285531-5A3A-4015-920E-F8FF5022E776}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1E10619-2BCF-4BA3-B155-7825AEEDFCE8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17224,5 +17239,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1E10619-2BCF-4BA3-B155-7825AEEDFCE8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E574B79-C17B-4CDE-A188-859CFF65AA1F}"/>
 </file>
</xml_diff>